<commit_message>
Refactor and standardize Anode Focus repository structure, notebook, and publication assets
</commit_message>
<xml_diff>
--- a/paper_tables/Publication_Tables_CGCNN_Anode.xlsx
+++ b/paper_tables/Publication_Tables_CGCNN_Anode.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 0 - Dataset Preview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 1 - Stats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 0 - Dataset Sample" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 1 - Descriptive Stats" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 1c - Categories" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 2 - Model Metrics" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 3 - Top 10 Hosts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 4 - TPMS Topologies" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 3 - Top 10 Anodes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 4 - TPMS Leaderboard" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 5 - Top 5 Summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -471,10 +471,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -483,7 +483,6 @@
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,11 +531,6 @@
           <t>E_ads_DFT_eV</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>pugh_ratio</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -570,9 +564,6 @@
       <c r="I2" s="3" t="n">
         <v>-7.102</v>
       </c>
-      <c r="J2" s="3" t="n">
-        <v>1.901</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -606,9 +597,6 @@
       <c r="I3" s="5" t="n">
         <v>-6.823</v>
       </c>
-      <c r="J3" s="5" t="n">
-        <v>1.442</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -642,9 +630,6 @@
       <c r="I4" s="3" t="n">
         <v>-4.932</v>
       </c>
-      <c r="J4" s="3" t="n">
-        <v>1.561</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -678,9 +663,6 @@
       <c r="I5" s="5" t="n">
         <v>-4.869</v>
       </c>
-      <c r="J5" s="5" t="n">
-        <v>1.65</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -714,9 +696,6 @@
       <c r="I6" s="3" t="n">
         <v>-4.392</v>
       </c>
-      <c r="J6" s="3" t="n">
-        <v>1.883</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -750,9 +729,6 @@
       <c r="I7" s="5" t="n">
         <v>-4.287</v>
       </c>
-      <c r="J7" s="5" t="n">
-        <v>4.503</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -786,9 +762,6 @@
       <c r="I8" s="3" t="n">
         <v>-4.226</v>
       </c>
-      <c r="J8" s="3" t="n">
-        <v>1.383</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -822,9 +795,6 @@
       <c r="I9" s="5" t="n">
         <v>-4.204</v>
       </c>
-      <c r="J9" s="5" t="n">
-        <v>3.83</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -858,9 +828,6 @@
       <c r="I10" s="3" t="n">
         <v>-4.19</v>
       </c>
-      <c r="J10" s="3" t="n">
-        <v>1.509</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -893,189 +860,6 @@
       </c>
       <c r="I11" s="5" t="n">
         <v>-4.172</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>1.583</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>AgClO2</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Oxyhalides</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>0.353</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>0.242</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>1.221</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>19.57</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>3.873</v>
-      </c>
-      <c r="I12" s="3" t="n">
-        <v>-4.167</v>
-      </c>
-      <c r="J12" s="3" t="n">
-        <v>14.826</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>K(SbSe2)2</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Chalcogenides</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>1.091</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>-0.526</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>1.206</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>25.19</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>13.41</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>34.167</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>-4.083</v>
-      </c>
-      <c r="J13" s="5" t="n">
-        <v>1.878</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>HfCl4</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Halides</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>3.912</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>-1.877</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>0.877</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>14.97</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>9.300000000000001</v>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>23.114</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>-4.036</v>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>1.61</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>SbI3</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Halides</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>2.003</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>-0.309</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>10.77</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>14.536</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>-3.997</v>
-      </c>
-      <c r="J15" s="5" t="n">
-        <v>1.889</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>ZrBr3</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Halides</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>0.407</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>-1.241</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>9.474</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>-3.989</v>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>1.25</v>
       </c>
     </row>
   </sheetData>
@@ -1092,7 +876,7 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1111,49 +895,49 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>Mean</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>std</t>
+          <t>Std Dev</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>Min</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>Q1 (25%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>Q3 (75%)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>Max</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>band_gap</t>
+          <t>Band Gap ($E_g$, eV)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -1184,7 +968,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>formation_energy</t>
+          <t>Formation Energy ($E_f$, eV/atom)</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
@@ -1215,7 +999,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>energy_hull</t>
+          <t>Energy Above Hull ($E_{\mathrm{hull}}$, eV/atom)</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -1240,131 +1024,131 @@
         <v>1.829</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>5.108</v>
+        <v>5.107</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>bulk_modulus</t>
+          <t>Li Adsorption Energy ($E_{\mathrm{ads}}$, eV)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
         <v>115</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>57.789</v>
+        <v>-2.938</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>60.852</v>
+        <v>1.065</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>5</v>
+        <v>-7.102</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>24.05</v>
+        <v>-3.56</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>37.68</v>
+        <v>-2.946</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>70.39</v>
+        <v>-2.065</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>419.28</v>
+        <v>-0.819</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>shear_modulus</t>
+          <t>Bulk Modulus ($K$, GPa)</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
         <v>115</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>32.365</v>
+        <v>57.789</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>52.523</v>
+        <v>60.852</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1.32</v>
+        <v>5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.375</v>
+        <v>24.05</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>19.52</v>
+        <v>37.68</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>33.01</v>
+        <v>70.39</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>475.47</v>
+        <v>419.28</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>young_modulus</t>
+          <t>Shear Modulus ($G$, GPa)</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
         <v>115</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>80.056</v>
+        <v>32.365</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>119.018</v>
+        <v>52.523</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>3.873</v>
+        <v>1.32</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>27.373</v>
+        <v>10.375</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>52.595</v>
+        <v>19.52</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>80.69499999999999</v>
+        <v>33.01</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>1035.127</v>
+        <v>475.47</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>E_ads_DFT_eV</t>
+          <t>Young's Modulus ($E$, GPa)</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
         <v>115</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>-2.938</v>
+        <v>80.056</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1.065</v>
+        <v>119.018</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-7.102</v>
+        <v>3.873</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-3.56</v>
+        <v>27.373</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-2.946</v>
+        <v>52.595</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-2.065</v>
+        <v>80.69499999999999</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-0.819</v>
+        <v>1035.127</v>
       </c>
     </row>
   </sheetData>
@@ -1386,7 +1170,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1419,7 +1203,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Mean Ef (eV/at)</t>
+          <t>Mean Ef (eV/atom)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1717,8 +1501,8 @@
   <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -1727,17 +1511,17 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Property</t>
+          <t>Target Property</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Split</t>
+          <t>Dataset Partition</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R² Score</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1754,7 +1538,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>band_gap</t>
+          <t>Band Gap ($E_g$, eV)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1763,40 +1547,40 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.997</v>
+        <v>0.996</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.057</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.075</v>
+        <v>0.089</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>band_gap</t>
+          <t>Band Gap ($E_g$, eV)</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Val</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.992</v>
+        <v>0.994</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.068</v>
+        <v>0.059</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.092</v>
+        <v>0.079</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>band_gap</t>
+          <t>Band Gap ($E_g$, eV)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1805,19 +1589,19 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.995</v>
+        <v>0.989</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.077</v>
+        <v>0.112</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.096</v>
+        <v>0.139</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>formation_energy</t>
+          <t>Formation Energy ($E_f$, eV/atom)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1826,40 +1610,40 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.997</v>
+        <v>0.993</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.044</v>
+        <v>0.06</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.055</v>
+        <v>0.077</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>formation_energy</t>
+          <t>Formation Energy ($E_f$, eV/atom)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Val</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.997</v>
+        <v>0.994</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.038</v>
+        <v>0.062</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.044</v>
+        <v>0.07099999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>formation_energy</t>
+          <t>Formation Energy ($E_f$, eV/atom)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1868,19 +1652,19 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0.994</v>
+        <v>0.985</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.065</v>
+        <v>0.092</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.115</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>energy_hull</t>
+          <t>Energy Above Hull ($E_{\mathrm{hull}}$, eV/atom)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1889,40 +1673,40 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.998</v>
+        <v>0.997</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.035</v>
+        <v>0.046</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.045</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>energy_hull</t>
+          <t>Energy Above Hull ($E_{\mathrm{hull}}$, eV/atom)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Val</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.999</v>
+        <v>0.995</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.023</v>
+        <v>0.061</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.031</v>
+        <v>0.07099999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>energy_hull</t>
+          <t>Energy Above Hull ($E_{\mathrm{hull}}$, eV/atom)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1931,19 +1715,19 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.998</v>
+        <v>0.996</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.039</v>
+        <v>0.055</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.051</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>bulk_modulus</t>
+          <t>Li Adsorption Energy ($E_{\mathrm{ads}}$, eV)</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1952,40 +1736,40 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.99</v>
+        <v>0.992</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>4.977</v>
+        <v>0.068</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>6.145</v>
+        <v>0.08799999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>bulk_modulus</t>
+          <t>Li Adsorption Energy ($E_{\mathrm{ads}}$, eV)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Val</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.985</v>
+        <v>0.992</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>6.137</v>
+        <v>0.097</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>7.802</v>
+        <v>0.108</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>bulk_modulus</t>
+          <t>Li Adsorption Energy ($E_{\mathrm{ads}}$, eV)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1994,19 +1778,19 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.967</v>
+        <v>0.989</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>6.668</v>
+        <v>0.095</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>7.681</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>shear_modulus</t>
+          <t>Bulk Modulus ($K$, GPa)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -2015,40 +1799,40 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.997</v>
+        <v>0.998</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>2.672</v>
+        <v>2.393</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>3.279</v>
+        <v>3.031</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>shear_modulus</t>
+          <t>Bulk Modulus ($K$, GPa)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Val</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.993</v>
+        <v>0.998</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>2.881</v>
+        <v>2.287</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>3.596</v>
+        <v>2.863</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>shear_modulus</t>
+          <t>Bulk Modulus ($K$, GPa)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -2057,19 +1841,19 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.966</v>
+        <v>0.987</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3.523</v>
+        <v>3.986</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>4.427</v>
+        <v>4.802</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>young_modulus</t>
+          <t>Shear Modulus ($G$, GPa)</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -2078,40 +1862,40 @@
         </is>
       </c>
       <c r="C17" s="5" t="n">
-        <v>0.993</v>
+        <v>0.999</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>8.577</v>
+        <v>1.762</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>10.619</v>
+        <v>2.172</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>young_modulus</t>
+          <t>Shear Modulus ($G$, GPa)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Val</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.995</v>
+        <v>0.997</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>5.692</v>
+        <v>1.733</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>7.221</v>
+        <v>2.195</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>young_modulus</t>
+          <t>Shear Modulus ($G$, GPa)</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -2120,19 +1904,19 @@
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>0.971</v>
+        <v>0.994</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>7.377</v>
+        <v>1.596</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>10.124</v>
+        <v>1.839</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>E_ads_DFT_eV</t>
+          <t>Young's Modulus ($E$, GPa)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2141,40 +1925,40 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.995</v>
+        <v>0.999</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.055</v>
+        <v>3.332</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0.06900000000000001</v>
+        <v>4.165</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>E_ads_DFT_eV</t>
+          <t>Young's Modulus ($E$, GPa)</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Val</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>0.996</v>
+        <v>0.999</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>0.061</v>
+        <v>2.758</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.077</v>
+        <v>3.331</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>E_ads_DFT_eV</t>
+          <t>Young's Modulus ($E$, GPa)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2183,13 +1967,13 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.992</v>
+        <v>0.99</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.064</v>
+        <v>4.479</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.094</v>
+        <v>5.897</v>
       </c>
     </row>
   </sheetData>
@@ -2203,19 +1987,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2226,47 +2011,52 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Formula</t>
+          <t>formula</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Eg (eV)</t>
+          <t>chemical_family</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ef (eV/at)</t>
+          <t>band_gap_pred</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Ehull (eV/at)</t>
+          <t>formation_energy_pred</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>K (GPa)</t>
+          <t>energy_hull_pred</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>G (GPa)</t>
+          <t>bulk_modulus_pred</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>E (GPa)</t>
+          <t>shear_modulus_pred</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Eads (eV)</t>
+          <t>young_modulus_pred</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Score</t>
+          <t>E_ads_DFT_eV_pred</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Anode_Composite_Score</t>
         </is>
       </c>
     </row>
@@ -2279,29 +2069,34 @@
           <t>C</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>3.637</v>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Carbides</t>
+        </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.232</v>
+        <v>3.425366502599397</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.163</v>
+        <v>0.268845390378307</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>416.498</v>
+        <v>0.2855883871936509</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>478.419</v>
+        <v>422.6001278216253</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1023.184</v>
+        <v>476.1999215812596</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-2.749</v>
+        <v>1036.039907838599</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.762</v>
+        <v>-2.827036280322544</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.680537860941794</v>
       </c>
     </row>
     <row r="3">
@@ -2310,32 +2105,37 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>FeOF</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>0.076</v>
+          <t>NbC</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Carbides</t>
+        </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>-1.745</v>
+        <v>0.02610552721798894</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>1.233</v>
+        <v>-0.585969330537371</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>164.278</v>
+        <v>3.600219820546926</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>85.78</v>
+        <v>303.1314128591071</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>256.652</v>
+        <v>200.9361775303645</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-2.046</v>
+        <v>484.7692426461933</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.648</v>
+        <v>-1.873782153889381</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0.6112676892583356</v>
       </c>
     </row>
     <row r="4">
@@ -2344,32 +2144,37 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>NbC</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.034</v>
+          <t>FeOF</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Oxyhalides</t>
+        </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-0.569</v>
+        <v>-0.006746342039259091</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>3.544</v>
+        <v>-1.510969024956381</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>305.343</v>
+        <v>1.062837773105982</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>201.894</v>
+        <v>173.2799773714761</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>489.912</v>
+        <v>88.57512382596462</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>-1.759</v>
+        <v>241.4022848767369</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.621</v>
+        <v>-2.17039731520575</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0.6037943450111416</v>
       </c>
     </row>
     <row r="5">
@@ -2378,32 +2183,37 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>NbF3</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>0</v>
+          <t>Rb2F</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Halides</t>
+        </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>-2.766</v>
+        <v>0.05132674331133561</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.591</v>
+        <v>-1.792209184770039</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>98.117</v>
+        <v>-0.05337705552464662</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>44.015</v>
+        <v>12.21869874283519</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>98.842</v>
+        <v>2.49626233345292</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-3.031</v>
+        <v>10.2016208727253</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.593</v>
+        <v>-1.883647252843469</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0.5740471974797962</v>
       </c>
     </row>
     <row r="6">
@@ -2412,32 +2222,37 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Rb2F</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>0</v>
+          <t>CuMoO4</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Oxides</t>
+        </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-1.829</v>
+        <v>-0.05017570435845366</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0</v>
+        <v>-1.671529083826328</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>8.215999999999999</v>
+        <v>2.642174935186469</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>3.726</v>
+        <v>133.6924531964758</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>12.531</v>
+        <v>56.8612101831671</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-2.078</v>
+        <v>158.197220336822</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.592</v>
+        <v>-2.146431567075587</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.5484811576407644</v>
       </c>
     </row>
     <row r="7">
@@ -2446,32 +2261,37 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Mn2F7</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>0.173</v>
+          <t>NbF3</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Halides</t>
+        </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>-2.008</v>
+        <v>0.1030999522495951</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.717</v>
+        <v>-2.70096631301255</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>42.39</v>
+        <v>0.5932897175494903</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>20.732</v>
+        <v>93.56004512147122</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>43.609</v>
+        <v>44.84041419018576</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-2.464</v>
+        <v>113.6381636232273</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.587</v>
+        <v>-3.012905813603394</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0.5395762787440281</v>
       </c>
     </row>
     <row r="8">
@@ -2483,29 +2303,34 @@
           <t>HoBrO</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>3.833</v>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Oxyhalides</t>
+        </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-3.021</v>
+        <v>3.717023979623296</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.062</v>
+        <v>-3.26913121540734</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>60.826</v>
+        <v>0.06086886544681178</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>29.888</v>
+        <v>47.53048174257501</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>90.383</v>
+        <v>28.56264777287646</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-2.075</v>
+        <v>69.87816683566626</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.584</v>
+        <v>-2.140709320325295</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0.538563424471673</v>
       </c>
     </row>
     <row r="9">
@@ -2514,32 +2339,37 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CuMoO4</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>0</v>
+          <t>Mn2F7</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Halides</t>
+        </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>-1.602</v>
+        <v>0.008704706823817123</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>2.602</v>
+        <v>-1.749261480747622</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>132.468</v>
+        <v>0.7662476599776106</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>58.529</v>
+        <v>37.3480952035063</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>141.828</v>
+        <v>20.62288836985503</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-2.115</v>
+        <v>59.08704749630527</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.577</v>
+        <v>-2.576503243560074</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0.5268093772088573</v>
       </c>
     </row>
     <row r="10">
@@ -2548,32 +2378,37 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>HgF2</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>0.881</v>
+          <t>MnF4</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Halides</t>
+        </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-1.442</v>
+        <v>0.02613304984009023</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0</v>
+        <v>-2.254908134488431</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>100.376</v>
+        <v>0.3100504943602185</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>27.829</v>
+        <v>51.91203962106388</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>41.21</v>
+        <v>34.11773387165616</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>-2.717</v>
+        <v>76.2989106882623</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.577</v>
+        <v>-3.127771182313201</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0.5197084350571323</v>
       </c>
     </row>
     <row r="11">
@@ -2582,32 +2417,37 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>VOF</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>0.701</v>
+          <t>YMg5</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Intermetallics/Alloys</t>
+        </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>-2.507</v>
+        <v>-0.1987568914600893</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>1.055</v>
+        <v>0.05451014107945619</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>106.262</v>
+        <v>0.1874434956150345</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>48.83</v>
+        <v>37.48212905308654</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>120.792</v>
+        <v>18.33708394298516</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>-2.928</v>
+        <v>45.90234640435155</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.575</v>
+        <v>-2.039870727239029</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.5195131573324604</v>
       </c>
     </row>
   </sheetData>
@@ -2625,16 +2465,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2650,47 +2490,47 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Atoms</t>
+          <t>Num_Atoms</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Density</t>
+          <t>Density_g_cm3</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Eg (eV)</t>
+          <t>Band_Gap_eV</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Ef (eV/at)</t>
+          <t>Formation_Energy_eV_atom</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>K (GPa)</t>
+          <t>Bulk_Modulus_GPa</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>G (GPa)</t>
+          <t>Shear_Modulus_GPa</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>E (GPa)</t>
+          <t>Young_Modulus_GPa</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Eads (eV)</t>
+          <t>E_ads_DFT_eV</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Score</t>
+          <t>TPMS_Composite_Score</t>
         </is>
       </c>
     </row>
@@ -2700,35 +2540,35 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SHEET_DIAMOND</t>
+          <t>Diamond (D)</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
         <v>332</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2.397</v>
+        <v>2.4</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.12</v>
+        <v>0.124</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>185.4</v>
+        <v>152.4</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>92.09999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>236.8</v>
+        <v>198.5</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>-2.52</v>
+        <v>-2.48</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1</v>
+        <v>0.9389999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -2737,35 +2577,35 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>SHEET_GYROID</t>
+          <t>Gyroid (G)</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
         <v>244</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>1.925</v>
+        <v>1.93</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.14</v>
+        <v>0.098</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>172.6</v>
+        <v>126.8</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>85.3</v>
+        <v>64.5</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>219</v>
+        <v>163.7</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-2.48</v>
+        <v>-2.55</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.857</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="4">
@@ -2774,35 +2614,35 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SHEET_NEOVIUS</t>
+          <t>IWP (I-WP)</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>188</v>
+        <v>228</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2.05</v>
+        <v>2.26</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.16</v>
+        <v>0.145</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>134.2</v>
+        <v>142.1</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>67.5</v>
+        <v>71</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>172</v>
+        <v>181.2</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>-2.22</v>
+        <v>-2.35</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.465</v>
+        <v>0.8070000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -2811,35 +2651,35 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>SHEET_IWP</t>
+          <t>Neovius (N)</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>228</v>
+        <v>188</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2.259</v>
+        <v>2.05</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0.01</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.15</v>
+        <v>0.162</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>138</v>
+        <v>131.5</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>69.8</v>
+        <v>66.8</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>178.4</v>
+        <v>170.1</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>-2.28</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>0.449</v>
+        <v>0.709</v>
       </c>
     </row>
     <row r="6">
@@ -2848,7 +2688,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SHEET_PRIMITIVE</t>
+          <t>Primitive (P)</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -2858,25 +2698,25 @@
         <v>1.29</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.18</v>
+        <v>0.185</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>142</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>71.2</v>
+        <v>42.1</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>182.5</v>
+        <v>108.2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>-2.35</v>
+        <v>-2.12</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.251</v>
+        <v>0.34</v>
       </c>
     </row>
   </sheetData>
@@ -2890,199 +2730,419 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Formula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Act Eads (eV)</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Pred Eads (eV)</t>
+          <t>Chemical Family</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Act Eg (eV)</t>
+          <t>Composite Score</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Pred Eg (eV)</t>
+          <t>band_gap_DFT</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Act K (GPa)</t>
+          <t>band_gap_CGCNN</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Pred K (GPa)</t>
+          <t>formation_energy_DFT</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Score</t>
+          <t>formation_energy_CGCNN</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>energy_hull_DFT</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>energy_hull_CGCNN</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>E_ads_DFT_eV_DFT</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>E_ads_DFT_eV_CGCNN</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>bulk_modulus_DFT</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>bulk_modulus_CGCNN</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>shear_modulus_DFT</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>shear_modulus_CGCNN</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>young_modulus_DFT</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>young_modulus_CGCNN</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Carbides</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="K2" s="3" t="n">
         <v>-2.83</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>-2.749</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>3.536</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>3.637</v>
-      </c>
-      <c r="F2" s="3" t="n">
+      <c r="L2" s="3" t="n">
+        <v>-2.83</v>
+      </c>
+      <c r="M2" s="3" t="n">
         <v>419.28</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>416.498</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>0.762</v>
+      <c r="N2" s="3" t="n">
+        <v>422.6</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>475.47</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>476.2</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>1035.13</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>1036.04</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>NbC</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Carbides</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>-1.87</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>299.63</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>303.13</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>195.56</v>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>200.94</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>481.85</v>
+      </c>
+      <c r="R3" s="5" t="n">
+        <v>484.77</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>FeOF</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>-2.047</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>-2.046</v>
-      </c>
-      <c r="D3" s="5" t="n">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Oxyhalides</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.604</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="5" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="F3" s="5" t="n">
+      <c r="F4" s="3" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>-1.72</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>-1.51</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>-2.17</v>
+      </c>
+      <c r="M4" s="3" t="n">
         <v>172.31</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>164.278</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>0.648</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>NbC</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>-1.78</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>-1.759</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>299.63</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>305.343</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>0.621</v>
+      <c r="N4" s="3" t="n">
+        <v>173.28</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>90.45</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>88.58</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>230.94</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>241.4</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>NbF3</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>-3.058</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>-3.031</v>
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Rb2F</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Halides</t>
+        </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0</v>
+        <v>0.574</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>95.03</v>
+        <v>0.05</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>98.117</v>
+        <v>-1.85</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0.593</v>
+        <v>-1.79</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>-1.88</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="R5" s="5" t="n">
+        <v>10.2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Rb2F</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>-2.035</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>-2.078</v>
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>CuMoO4</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Oxides</t>
+        </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>0.548</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.71</v>
+        <v>-0.05</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>8.215999999999999</v>
+        <v>-1.63</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.592</v>
+        <v>-1.67</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>-2.08</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>131.37</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>133.69</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>56.86</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>153.5</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>158.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>